<commit_message>
Data set para cargar
</commit_message>
<xml_diff>
--- a/Semana_1/colcap_semana1.xlsx
+++ b/Semana_1/colcap_semana1.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7B2D9BB-058B-4C8F-A170-7092557BFF7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B36964E-4381-42CF-9E48-9F2D17334564}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9117" uniqueCount="9003">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9116" uniqueCount="9002">
   <si>
     <t>Índice</t>
   </si>
@@ -26980,9 +26980,6 @@
   </si>
   <si>
     <t/>
-  </si>
-  <si>
-    <t>Descargado de sistema del Banco de la República sábado, 3 de octubre de 2026 4:06:03 p. m.</t>
   </si>
   <si>
     <t>Nombre de la serie</t>
@@ -27418,7 +27415,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B4553"/>
+  <dimension ref="A1:B4552"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -27427,10 +27424,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>9002</v>
+        <v>9001</v>
       </c>
       <c r="B1" t="s">
-        <v>9001</v>
+        <v>9000</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -63833,11 +63830,6 @@
     <row r="4552" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4552" t="s">
         <v>8987</v>
-      </c>
-    </row>
-    <row r="4553" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4553" t="s">
-        <v>8988</v>
       </c>
     </row>
   </sheetData>
@@ -63860,30 +63852,30 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>8988</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>8989</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>8990</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>8991</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>8992</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>8993</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>8994</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>8995</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>8996</v>
+        <v>8995</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>0</v>
@@ -63892,16 +63884,16 @@
         <v>8987</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>8996</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>8997</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>8998</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>8999</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>9000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>